<commit_message>
update observation vs a9aa2e624c1684f1f579bb019379fd5ed3dd0617
</commit_message>
<xml_diff>
--- a/nr-refacto-errors/ig/ValueSet-fr-core-vs-heartrate-body-location.xlsx
+++ b/nr-refacto-errors/ig/ValueSet-fr-core-vs-heartrate-body-location.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-06T14:44:44+00:00</t>
+    <t>2025-07-06T14:51:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -189,7 +189,7 @@
     <t>Structure of left radial artery (body structure)</t>
   </si>
   <si>
-    <t>24781000205105</t>
+    <t>1268741004</t>
   </si>
   <si>
     <t>Structure of left superficial temporal artery (body structure)</t>
@@ -261,7 +261,7 @@
     <t>Structure of right pulmonary artery (body structure)</t>
   </si>
   <si>
-    <t>24791000205107</t>
+    <t>1268742006</t>
   </si>
   <si>
     <t>Structure of right superficial temporal artery (body structure)</t>

</xml_diff>